<commit_message>
Adding artwork from final files before manufacture
git-svn-id: https://svn2.phy.bris.ac.uk/svn/uob-hep-pc049a/trunk@20 e1591323-3689-4d5a-aa31-d1a7cbdc5706
</commit_message>
<xml_diff>
--- a/www/Docs/pc049a_checklist.xlsx
+++ b/www/Docs/pc049a_checklist.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
   <si>
     <t>General checks:</t>
   </si>
@@ -96,6 +96,27 @@
   </si>
   <si>
     <t>Clock circuitry looks OK.</t>
+  </si>
+  <si>
+    <t>PCB Checks</t>
+  </si>
+  <si>
+    <t>pc049a_toplevel_40_a16-5_ans.brd</t>
+  </si>
+  <si>
+    <t>No DRC</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>No unplaced</t>
+  </si>
+  <si>
+    <t>No unconnected</t>
+  </si>
+  <si>
+    <t>No dangling</t>
   </si>
 </sst>
 </file>
@@ -110,6 +131,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -193,10 +215,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
-    <tabColor rgb="00FFFFFF"/>
+    <tabColor rgb="FFFFFFFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr defaultRowHeight="12.8"/>
   <cols>
     <col collapsed="false" hidden="false" max="1" min="1" style="0" width="55.4285714285714"/>
@@ -325,6 +347,46 @@
         <v>26</v>
       </c>
     </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="B37" s="0" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Checking in files before copying to GIT
git-svn-id: https://svn2.phy.bris.ac.uk/svn/uob-hep-pc049a/trunk@26 e1591323-3689-4d5a-aa31-d1a7cbdc5706
</commit_message>
<xml_diff>
--- a/www/Docs/pc049a_checklist.xlsx
+++ b/www/Docs/pc049a_checklist.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="61">
   <si>
     <t>General checks:</t>
   </si>
@@ -98,12 +98,36 @@
     <t>Clock circuitry looks OK.</t>
   </si>
   <si>
+    <t>Check configuration </t>
+  </si>
+  <si>
+    <t>JTAG to FPGA pins</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>M0 , M1 = high , low</t>
+  </si>
+  <si>
+    <t>Done , program pulled high</t>
+  </si>
+  <si>
+    <t>JTAG to programming header</t>
+  </si>
+  <si>
+    <t>SPI to FPGA</t>
+  </si>
+  <si>
     <t>PCB Checks</t>
   </si>
   <si>
     <t>pc049a_toplevel_40_a16-5_ans.brd</t>
   </si>
   <si>
+    <t>pc049a_toplevel_47.brd</t>
+  </si>
+  <si>
     <t>No DRC</t>
   </si>
   <si>
@@ -117,6 +141,63 @@
   </si>
   <si>
     <t>No dangling</t>
+  </si>
+  <si>
+    <t>good enough – some dangling vias</t>
+  </si>
+  <si>
+    <t>Stack up</t>
+  </si>
+  <si>
+    <t>Diff pairs on 1 Gbit/s tracks = 0.130mm tracks / 0.200mm gap</t>
+  </si>
+  <si>
+    <t>good enough. 0.127mm with 0.18mm gap = 98 ohms</t>
+  </si>
+  <si>
+    <t>silk screen top</t>
+  </si>
+  <si>
+    <t>silk screen bottom</t>
+  </si>
+  <si>
+    <t>drill figure</t>
+  </si>
+  <si>
+    <t>done</t>
+  </si>
+  <si>
+    <t>padstacks</t>
+  </si>
+  <si>
+    <t>Warning – via annular ring too small....</t>
+  </si>
+  <si>
+    <t>All layers checked</t>
+  </si>
+  <si>
+    <t>good enough</t>
+  </si>
+  <si>
+    <t>delete islands</t>
+  </si>
+  <si>
+    <t>Ok – none shown in datasheet</t>
+  </si>
+  <si>
+    <t>Check power supply – DRVCC decoupling??</t>
+  </si>
+  <si>
+    <t>Double check RFB</t>
+  </si>
+  <si>
+    <t>Gloss radius corners</t>
+  </si>
+  <si>
+    <t>Gloss filet pads</t>
+  </si>
+  <si>
+    <t>current pc049a_toplevel_49.brd</t>
   </si>
 </sst>
 </file>
@@ -157,12 +238,19 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double"/>
       <diagonal/>
     </border>
   </borders>
@@ -191,12 +279,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -218,11 +310,12 @@
     <tabColor rgb="FFFFFFFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N82"/>
   <sheetFormatPr defaultRowHeight="12.8"/>
   <cols>
     <col collapsed="false" hidden="false" max="1" min="1" style="0" width="55.4285714285714"/>
-    <col collapsed="false" hidden="false" max="11" min="2" style="0" width="11.5204081632653"/>
+    <col collapsed="false" hidden="false" max="2" min="2" style="0" width="31.030612244898"/>
+    <col collapsed="false" hidden="false" max="11" min="3" style="0" width="11.5204081632653"/>
     <col collapsed="false" hidden="false" max="12" min="12" style="0" width="20.7244897959184"/>
     <col collapsed="false" hidden="false" max="13" min="13" style="0" width="23.8316326530612"/>
     <col collapsed="false" hidden="false" max="1025" min="14" style="0" width="11.5204081632653"/>
@@ -347,44 +440,194 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B36" s="0" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="B39" s="0" t="s">
+      <c r="C36" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="0" t="s">
         <v>30</v>
       </c>
+      <c r="C38" s="0" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="B40" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="B40" s="0" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="C40" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="B41" s="0" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="C42" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="B42" s="0" t="s">
-        <v>30</v>
+      <c r="C44" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="B49" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C49" s="0" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C51" s="0" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="B52" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C52" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B53" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C53" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C54" s="0" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C57" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="C59" s="0" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C61" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="C62" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="C64" s="0" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="C66" s="0" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C70" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C73" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="0" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="0" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="0" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="0" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="0" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>